<commit_message>
R05: diagnóstico NEREUS × SEEG final (bases na convenção do SEEG, critério SCN único, casamento concorrente do S19 e risco de dupla contagem na E4)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CWPuQS1EQNnCbSqHfPPCuA
</commit_message>
<xml_diff>
--- a/resultados/rodada05/diagnostico_seeg_nereus.xlsx
+++ b/resultados/rodada05/diagnostico_seeg_nereus.xlsx
@@ -543,7 +543,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Casamento concorrente: A busca também encontrou S19-RS ≈ Produção de combustíveis › Produção de combustíveis › Refino de petróleo + Química › Industrial › Química (0.071%, sentido 'não'), que usa as mesmas emissões do refino; ao todo, 16 combinações abaixo de 0.1% em outros setores usam 'Produção de combustíveis › Produção de combustíveis › Refino de petróleo' (10 no S19). As duas leituras se excluem: as 1736.0 mil t do refino não podem estar ao mesmo tempo no S38 e no S19. E, se o refino estiver no S38, as 2693.9 mil t do S19-RS (Refino de petróleo e coquerias) da NEREUS não têm contrapartida no SEEG do RS, cujas únicas unidades de refino ou coqueria são Agricultura › Solos manejados › Redução do estoque de C no solo; Geração de eletricidade › Produção de combustíveis › Refino de petróleo; Pecuária › Solos manejados › Redução do estoque de C no solo; Produção de combustíveis › Produção de combustíveis › Refino de petróleo (1812.1 mil t, ambas usadas na hipótese do S38). Isso enfraquece o indício e é um risco para a E4: se o S19 da NEREUS já contiver o refino, a E4 o conta duas vezes no S19-RS (2693.9 + 1812.1 = 4506.0 mil t); vale tratá-lo como sensibilidade.</t>
+          <t>Casamento concorrente: A busca também encontrou S19-RS ≈ Produção de combustíveis › Produção de combustíveis › Refino de petróleo + Química › Industrial › Química (0.071%, sentido 'não'), que usa as mesmas emissões do refino; ao todo, 16 combinações abaixo de 0.1% em outros setores usam 'Produção de combustíveis › Produção de combustíveis › Refino de petróleo' (10 no S19). As duas leituras se excluem: as 1736.0 mil t do refino não podem estar ao mesmo tempo no S38 e no S19. E, se o refino estiver no S38, as 2693.9 mil t do S19-RS (Refino de petróleo e coquerias) da NEREUS não têm contrapartida no SEEG do RS, cujas únicas unidades de refino ou coqueria são Geração de eletricidade › Produção de combustíveis › Refino de petróleo; Produção de combustíveis › Produção de combustíveis › Refino de petróleo (1812.1 mil t, ambas usadas na hipótese do S38). Isso enfraquece o indício e é um risco para a E4: se o S19 da NEREUS já contiver o refino, a E4 o conta duas vezes no S19-RS (2693.9 + 1812.1 = 4506.0 mil t); vale tratá-lo como sensibilidade.</t>
         </is>
       </c>
     </row>
@@ -37492,7 +37492,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>4. Casamentos no RS: 84982 combinações por setor (1, 2 ou 3 unidades de um mesmo tipo) × 8 setores (7 + o controle S38) = 679856 testes. Com |dif| &lt; 0.1%: 224 combinações (126 núcleos distintos depois de tirar as unidades desprezíveis, |valor| &lt; 0.1% do alvo, que geram quase repetições). Por acaso seriam esperadas da ordem de 211 (heurística de densidade uniforme: nº em ±5% ÷ 50; por setor erra até ~3 vezes, ver contagens). Pelo critério SCN, aplicado igual a todos os setores, 0 têm sentido econômico 'sim' e 9 'discutível'; as demais não têm sentido econômico.</t>
+          <t>4. Casamentos no RS: 84982 combinações por setor (1, 2 ou 3 unidades de um mesmo tipo) × 8 setores (7 + o controle S38) = 679856 testes. Com |dif| &lt; 0.1%: 224 combinações (126 núcleos distintos depois de tirar as unidades desprezíveis, |valor| &lt; 0.1% do alvo, que geram quase repetições). Por acaso seriam esperadas da ordem de 211 (heurística de densidade uniforme: nº em ±5% ÷ 50; por setor erra até ~3 vezes, ver contagens). Pelo critério SCN, aplicado igual a todos os setores, 0 têm sentido econômico 'sim' e 9 'discutível'; as demais não têm sentido econômico. 9 'discutível' no S01, todas com 'Agricultura › Alterações de uso da terra › Desmatamento' (25938.8 mil t, -1.0% do S01 sozinha) mais unidades pequenas: só MUT e fragmentos, não a atividade.</t>
         </is>
       </c>
     </row>
@@ -37506,7 +37506,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>6. Casamento concorrente. A busca também encontrou S19-RS ≈ Produção de combustíveis › Produção de combustíveis › Refino de petróleo + Química › Industrial › Química (0.071%, sentido 'não'), que usa as mesmas emissões do refino; ao todo, 16 combinações abaixo de 0.1% em outros setores usam 'Produção de combustíveis › Produção de combustíveis › Refino de petróleo' (10 no S19). As duas leituras se excluem: as 1736.0 mil t do refino não podem estar ao mesmo tempo no S38 e no S19. E, se o refino estiver no S38, as 2693.9 mil t do S19-RS (Refino de petróleo e coquerias) da NEREUS não têm contrapartida no SEEG do RS, cujas únicas unidades de refino ou coqueria são Agricultura › Solos manejados › Redução do estoque de C no solo; Geração de eletricidade › Produção de combustíveis › Refino de petróleo; Pecuária › Solos manejados › Redução do estoque de C no solo; Produção de combustíveis › Produção de combustíveis › Refino de petróleo (1812.1 mil t, ambas usadas na hipótese do S38). Isso enfraquece o indício e é um risco para a E4: se o S19 da NEREUS já contiver o refino, a E4 o conta duas vezes no S19-RS (2693.9 + 1812.1 = 4506.0 mil t); vale tratá-lo como sensibilidade.</t>
+          <t>6. Casamento concorrente. A busca também encontrou S19-RS ≈ Produção de combustíveis › Produção de combustíveis › Refino de petróleo + Química › Industrial › Química (0.071%, sentido 'não'), que usa as mesmas emissões do refino; ao todo, 16 combinações abaixo de 0.1% em outros setores usam 'Produção de combustíveis › Produção de combustíveis › Refino de petróleo' (10 no S19). As duas leituras se excluem: as 1736.0 mil t do refino não podem estar ao mesmo tempo no S38 e no S19. E, se o refino estiver no S38, as 2693.9 mil t do S19-RS (Refino de petróleo e coquerias) da NEREUS não têm contrapartida no SEEG do RS, cujas únicas unidades de refino ou coqueria são Geração de eletricidade › Produção de combustíveis › Refino de petróleo; Produção de combustíveis › Produção de combustíveis › Refino de petróleo (1812.1 mil t, ambas usadas na hipótese do S38). Isso enfraquece o indício e é um risco para a E4: se o S19 da NEREUS já contiver o refino, a E4 o conta duas vezes no S19-RS (2693.9 + 1812.1 = 4506.0 mil t); vale tratá-lo como sensibilidade.</t>
         </is>
       </c>
     </row>

</xml_diff>